<commit_message>
Añade .nojekyll para desactivar Jekyll en GitHub Pages
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Negocio Maduro FY27.xlsx
+++ b/Negocio Maduro FY27.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/angelrodmen/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{89182E86-2BDD-A946-9E81-5EF1ED1949DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE0496BE-3503-7D40-8362-45E7F3B1E552}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5180" yWindow="1880" windowWidth="28040" windowHeight="17180" xr2:uid="{C24AFCBA-2F5F-514C-AB35-9A128891F327}"/>
+    <workbookView xWindow="-38400" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{C24AFCBA-2F5F-514C-AB35-9A128891F327}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="SAN CIB" sheetId="2" r:id="rId2"/>
+    <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="93">
   <si>
     <t>3.1 BBVA CIB</t>
   </si>
@@ -232,9 +234,6 @@
     <t>Casis de USO IA delsde los CoE para areas de negocio.</t>
   </si>
   <si>
-    <t>3.2 SAN CIB</t>
-  </si>
-  <si>
     <t>OBJT FY27 - 26MM € y +350 Ftes que supone x2 desde 2025 (CIB+Geografías)</t>
   </si>
   <si>
@@ -271,13 +270,7 @@
     <t>Contexto de reducción de costes del 25-30%</t>
   </si>
   <si>
-    <t>Aplica también a T&amp;O</t>
-  </si>
-  <si>
     <t>Plan de adopción de IA y búsqueda de eficiencia</t>
-  </si>
-  <si>
-    <t>Aplica también a T&amp;O y ya nos están pidiendo contabilizar la eficiencia en los desarrollos</t>
   </si>
   <si>
     <t>Conseguir ser el primer proveedor en todos los dominios vs concentración global</t>
@@ -289,31 +282,52 @@
     <t>Conjugar la aplicación de IA en la externalización de servicios de Operaciones</t>
   </si>
   <si>
-    <t>Plan de impulso en FinCrime</t>
-  </si>
-  <si>
     <t>Plan CDAIO - conseguir ser agente de cambio en el plan de adopción en conjunción con Negocio</t>
-  </si>
-  <si>
-    <t>Plan de impulso en GDF y su derivada en BDH</t>
   </si>
   <si>
     <t>Planes de Data para los DataLakes (CoE BigData + BDH)</t>
   </si>
   <si>
-    <t>Plan de impulso en Finance</t>
-  </si>
-  <si>
     <t>Plan de posicionamiento en la primera línea de SDS</t>
   </si>
   <si>
-    <t>Plan de impulso en Accounting</t>
+    <t>Plan de impulso en FinCrime, GDF, Finance y Accounting (¿Quién?)</t>
   </si>
   <si>
-    <t>Priorización de ámbitos de crecimiento + establecimiento de aceleradores de capacidad</t>
+    <t>Planes para retomar senda alcista en branches (¿Cómo?)</t>
   </si>
   <si>
-    <t>Planes para retomar senda alcista en branches</t>
+    <t>Traer la experiencia de BBVA CIB Eng (Apoyo Antonio + Liderzago nueva etapa Daniel L. )</t>
+  </si>
+  <si>
+    <t>IA que se tiene que contabilizar la eficiencia en los desarrollos</t>
+  </si>
+  <si>
+    <t>CONTEXTO PLAN</t>
+  </si>
+  <si>
+    <t>GEOGRAFIAS (Actual X Ftes)</t>
+  </si>
+  <si>
+    <t>USA Muchas cosas proveedor 1</t>
+  </si>
+  <si>
+    <t>Mexico blalbalbalblab</t>
+  </si>
+  <si>
+    <t>Brasil dando caña con Vulcano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entender bien San Brasil Vulcano </t>
+  </si>
+  <si>
+    <t>Mexico XXXXX</t>
+  </si>
+  <si>
+    <t>Accion 1</t>
+  </si>
+  <si>
+    <t>Accion 2</t>
   </si>
 </sst>
 </file>
@@ -1164,13 +1178,13 @@
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="D33" s="2">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="E33" s="2">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
@@ -1181,13 +1195,13 @@
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2">
-        <v>400</v>
+        <v>517</v>
       </c>
       <c r="D34" s="2">
-        <v>550</v>
+        <v>634</v>
       </c>
       <c r="E34" s="2">
-        <v>685</v>
+        <v>754</v>
       </c>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
@@ -1215,7 +1229,7 @@
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
       <c r="E36" s="3">
-        <v>0.6</v>
+        <v>0.35</v>
       </c>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
@@ -1701,9 +1715,7 @@
     <row r="73" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
-      <c r="C73" s="1" t="s">
-        <v>61</v>
-      </c>
+      <c r="C73" s="1"/>
       <c r="D73" s="2"/>
       <c r="E73" s="2"/>
       <c r="F73" s="2"/>
@@ -1725,9 +1737,7 @@
     <row r="75" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
-      <c r="C75" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="C75" s="1"/>
       <c r="D75" s="2"/>
       <c r="E75" s="2"/>
       <c r="F75" s="2"/>
@@ -1737,12 +1747,8 @@
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A76" s="2"/>
-      <c r="B76" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C76" s="2" t="s">
-        <v>62</v>
-      </c>
+      <c r="B76" s="1"/>
+      <c r="C76" s="2"/>
       <c r="D76" s="2"/>
       <c r="E76" s="2"/>
       <c r="F76" s="2"/>
@@ -1752,12 +1758,8 @@
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A77" s="2"/>
-      <c r="B77" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C77" s="2" t="s">
-        <v>63</v>
-      </c>
+      <c r="B77" s="1"/>
+      <c r="C77" s="2"/>
       <c r="D77" s="2"/>
       <c r="E77" s="2"/>
       <c r="F77" s="2"/>
@@ -1767,12 +1769,8 @@
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A78" s="2"/>
-      <c r="B78" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C78" s="2" t="s">
-        <v>64</v>
-      </c>
+      <c r="B78" s="1"/>
+      <c r="C78" s="2"/>
       <c r="D78" s="2"/>
       <c r="E78" s="2"/>
       <c r="F78" s="2"/>
@@ -1794,12 +1792,8 @@
     <row r="80" spans="1:9" ht="19" x14ac:dyDescent="0.2">
       <c r="A80" s="2"/>
       <c r="B80" s="2"/>
-      <c r="C80" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D80" s="5" t="s">
-        <v>66</v>
-      </c>
+      <c r="C80" s="4"/>
+      <c r="D80" s="5"/>
       <c r="E80" s="2"/>
       <c r="F80" s="2"/>
       <c r="G80" s="2"/>
@@ -1808,15 +1802,9 @@
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A81" s="2"/>
-      <c r="B81" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C81" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D81" s="2" t="s">
-        <v>68</v>
-      </c>
+      <c r="B81" s="1"/>
+      <c r="C81" s="2"/>
+      <c r="D81" s="2"/>
       <c r="E81" s="2"/>
       <c r="F81" s="2"/>
       <c r="G81" s="2"/>
@@ -1826,12 +1814,8 @@
     <row r="82" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A82" s="2"/>
       <c r="B82" s="2"/>
-      <c r="C82" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>70</v>
-      </c>
+      <c r="C82" s="2"/>
+      <c r="D82" s="2"/>
       <c r="E82" s="2"/>
       <c r="F82" s="2"/>
       <c r="G82" s="2"/>
@@ -1841,12 +1825,8 @@
     <row r="83" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
-      <c r="C83" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D83" s="2" t="s">
-        <v>72</v>
-      </c>
+      <c r="C83" s="2"/>
+      <c r="D83" s="2"/>
       <c r="E83" s="2"/>
       <c r="F83" s="2"/>
       <c r="G83" s="2"/>
@@ -1866,15 +1846,9 @@
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A85" s="2"/>
-      <c r="B85" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C85" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="D85" s="6" t="s">
-        <v>74</v>
-      </c>
+      <c r="B85" s="1"/>
+      <c r="C85" s="6"/>
+      <c r="D85" s="6"/>
       <c r="E85" s="2"/>
       <c r="F85" s="2"/>
       <c r="G85" s="2"/>
@@ -1884,12 +1858,8 @@
     <row r="86" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
-      <c r="C86" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="D86" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="C86" s="6"/>
+      <c r="D86" s="2"/>
       <c r="E86" s="2"/>
       <c r="F86" s="2"/>
       <c r="G86" s="2"/>
@@ -1899,12 +1869,8 @@
     <row r="87" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
-      <c r="C87" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D87" s="2" t="s">
-        <v>78</v>
-      </c>
+      <c r="C87" s="2"/>
+      <c r="D87" s="2"/>
       <c r="E87" s="2"/>
       <c r="F87" s="2"/>
       <c r="G87" s="2"/>
@@ -1915,9 +1881,7 @@
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
-      <c r="D88" s="6" t="s">
-        <v>79</v>
-      </c>
+      <c r="D88" s="6"/>
       <c r="E88" s="2"/>
       <c r="F88" s="2"/>
       <c r="G88" s="2"/>
@@ -1937,15 +1901,9 @@
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A90" s="2"/>
-      <c r="B90" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C90" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D90" s="2" t="s">
-        <v>81</v>
-      </c>
+      <c r="B90" s="1"/>
+      <c r="C90" s="2"/>
+      <c r="D90" s="2"/>
       <c r="E90" s="2"/>
       <c r="F90" s="2"/>
       <c r="G90" s="2"/>
@@ -1955,12 +1913,8 @@
     <row r="91" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
-      <c r="C91" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D91" s="2" t="s">
-        <v>83</v>
-      </c>
+      <c r="C91" s="2"/>
+      <c r="D91" s="2"/>
       <c r="E91" s="2"/>
       <c r="F91" s="2"/>
       <c r="G91" s="2"/>
@@ -1970,12 +1924,8 @@
     <row r="92" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
-      <c r="C92" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D92" s="2" t="s">
-        <v>85</v>
-      </c>
+      <c r="C92" s="2"/>
+      <c r="D92" s="2"/>
       <c r="E92" s="2"/>
       <c r="F92" s="2"/>
       <c r="G92" s="2"/>
@@ -1985,12 +1935,8 @@
     <row r="93" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
-      <c r="C93" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="D93" s="2" t="s">
-        <v>87</v>
-      </c>
+      <c r="C93" s="2"/>
+      <c r="D93" s="2"/>
       <c r="E93" s="2"/>
       <c r="F93" s="2"/>
       <c r="G93" s="2"/>
@@ -2000,9 +1946,7 @@
     <row r="94" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
-      <c r="C94" s="6" t="s">
-        <v>88</v>
-      </c>
+      <c r="C94" s="6"/>
       <c r="D94" s="2"/>
       <c r="E94" s="2"/>
       <c r="F94" s="2"/>
@@ -11979,4 +11923,287 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6F48740-6088-694A-A2CC-2684BA3E3643}">
+  <dimension ref="B1:D46"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="75.33203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="4" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B2" s="2"/>
+      <c r="C2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B3" s="2"/>
+      <c r="C3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="B5" s="2"/>
+      <c r="C5" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B7" s="2"/>
+      <c r="C7" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B8" s="2"/>
+      <c r="C8" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B11" s="2"/>
+      <c r="C11" s="6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B12" s="2"/>
+      <c r="C12" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B15" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B16" s="2"/>
+      <c r="C16" s="6" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+    </row>
+    <row r="19" spans="2:4" ht="18" x14ac:dyDescent="0.2">
+      <c r="B19" s="2"/>
+      <c r="C19" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D19" s="2"/>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B20" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D20" s="2"/>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B21" s="2"/>
+      <c r="C21" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D21" s="2"/>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B22" s="2"/>
+      <c r="C22" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D22" s="2"/>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B24" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B25" s="2"/>
+      <c r="C25" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B26" s="2"/>
+      <c r="C26" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B27" s="2"/>
+      <c r="C27" s="6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="28" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+    </row>
+    <row r="29" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B29" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="30" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="C30" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="31" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="C31" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="32" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="C32" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="C35" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B36" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C36" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B37" s="2"/>
+      <c r="C37" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="38" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B38" s="2"/>
+      <c r="C38" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="39" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B39" s="2"/>
+    </row>
+    <row r="40" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B40" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C40" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="41" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B41" s="2"/>
+      <c r="C41" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="42" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B42" s="2"/>
+    </row>
+    <row r="43" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B43" s="2"/>
+    </row>
+    <row r="44" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B44" s="2"/>
+    </row>
+    <row r="45" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B45" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C45" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="46" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="C46" t="s">
+        <v>92</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DE9DEEF-B2FB-0F4D-8FA7-6C1E67DF60A7}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>